<commit_message>
update quotation example Excel files, README, and data documentation for office alignment guide
</commit_message>
<xml_diff>
--- a/常見的AI應用/office辦公室應用進階的對齊/報價單_示範成果_客戶2_遠景智慧製造(長備註測試).xlsx
+++ b/常見的AI應用/office辦公室應用進階的對齊/報價單_示範成果_客戶2_遠景智慧製造(長備註測試).xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G30"/>
+  <dimension ref="A2:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -621,7 +621,7 @@
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>AI 基礎與提示詞實作</t>
+          <t>AI 基礎觀念與提示詞工程實作</t>
         </is>
       </c>
       <c r="D13" s="16" t="n">
@@ -647,11 +647,11 @@
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>Excel 自動化工作坊</t>
+          <t>Python 與 Excel 辦公自動化工作坊</t>
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
@@ -673,19 +673,19 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>教材與課後諮詢</t>
+          <t>企業私有知識庫 RAG 系統架構評估</t>
         </is>
       </c>
       <c r="D15" s="16" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>人</t>
+          <t>式</t>
         </is>
       </c>
       <c r="F15" s="28" t="n">
-        <v>600</v>
+        <v>35000</v>
       </c>
       <c r="G15" s="49">
         <f>IF(AND(ISNUMBER(D13),ISNUMBER(F13)),D13*F13,"待填資料")</f>
@@ -694,111 +694,163 @@
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" t="inlineStr"/>
-      <c r="C16" s="52" t="n"/>
-      <c r="D16" s="52" t="n"/>
-      <c r="E16" s="52" t="n"/>
-      <c r="F16" s="53" t="n"/>
-      <c r="G16" s="49" t="n"/>
+      <c r="B16" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>教材版權與課後線上諮詢服務</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>人</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="n">
+        <v>600</v>
+      </c>
+      <c r="G16" s="49">
+        <f>IF(AND(ISNUMBER(D13),ISNUMBER(F13)),D13*F13,"待填資料")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="32" customHeight="1">
-      <c r="F17" s="30" t="inlineStr">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>實戰成果發表會與結業評審</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>場</t>
+        </is>
+      </c>
+      <c r="F17" s="28" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G17" s="49">
+        <f>IF(AND(ISNUMBER(D13),ISNUMBER(F13)),D13*F13,"待填資料")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" t="inlineStr"/>
+      <c r="C18" s="52" t="n"/>
+      <c r="D18" s="52" t="n"/>
+      <c r="E18" s="52" t="n"/>
+      <c r="F18" s="53" t="n"/>
+      <c r="G18" s="49" t="n"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="F19" s="30" t="inlineStr">
         <is>
           <t>未稅合計</t>
         </is>
       </c>
-      <c r="G17" s="50">
+      <c r="G19" s="50">
         <f>SUM(G13:G14)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="F18" s="30" t="inlineStr">
+    <row r="20">
+      <c r="F20" s="30" t="inlineStr">
         <is>
           <t>營業稅 5%</t>
         </is>
       </c>
-      <c r="G18" s="50">
+      <c r="G20" s="50">
         <f>G15*5%</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="F19" s="31" t="inlineStr">
+    <row r="21">
+      <c r="F21" s="31" t="inlineStr">
         <is>
           <t>含稅總計</t>
         </is>
       </c>
-      <c r="G19" s="51">
+      <c r="G21" s="51">
         <f>G15+G16</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="22" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>專案備註與付款條件</t>
         </is>
       </c>
-      <c r="C22" s="1" t="n"/>
-      <c r="D22" s="1" t="n"/>
-      <c r="E22" s="1" t="n"/>
-      <c r="F22" s="1" t="n"/>
-      <c r="G22" s="1" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="45" t="inlineStr">
+      <c r="C24" s="1" t="n"/>
+      <c r="D24" s="1" t="n"/>
+      <c r="E24" s="1" t="n"/>
+      <c r="F24" s="1" t="n"/>
+      <c r="G24" s="1" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="45" t="inlineStr">
         <is>
           <t>課程包含實作練習、範例檔案及課後問答。訓練完成並收到發票後 30 日內付款。此欄刻意使用較長文字，以測試合併儲存格換行及垂直對齊。</t>
         </is>
       </c>
-      <c r="C23" s="1" t="n"/>
-      <c r="D23" s="1" t="n"/>
-      <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="n"/>
-      <c r="G23" s="1" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="1" t="n"/>
-      <c r="G24" s="1" t="n"/>
-    </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="B25" s="1" t="n"/>
       <c r="C25" s="1" t="n"/>
       <c r="D25" s="1" t="n"/>
       <c r="E25" s="1" t="n"/>
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
     </row>
-    <row r="28">
-      <c r="B28" s="15" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="1" t="n"/>
+      <c r="G26" s="1" t="n"/>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="n"/>
+      <c r="E27" s="1" t="n"/>
+      <c r="F27" s="1" t="n"/>
+      <c r="G27" s="1" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>報價有效期限：2026/11/15</t>
         </is>
       </c>
-      <c r="C28" s="1" t="n"/>
-      <c r="D28" s="1" t="n"/>
-      <c r="E28" s="1" t="n"/>
-      <c r="F28" s="1" t="n"/>
-      <c r="G28" s="1" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="47" t="n"/>
+      <c r="C30" s="1" t="n"/>
+      <c r="D30" s="1" t="n"/>
+      <c r="E30" s="1" t="n"/>
+      <c r="F30" s="1" t="n"/>
+      <c r="G30" s="1" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="47" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B24:G24"/>
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B25:G27"/>
     <mergeCell ref="B2:G3"/>
     <mergeCell ref="D9:G9"/>
-    <mergeCell ref="B28:G28"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="D5:G5"/>
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="D6:G6"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D7:G7"/>
-    <mergeCell ref="B23:G25"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="B30:G30"/>
     <mergeCell ref="B8:C8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>